<commit_message>
Updated changes with new test user setup
</commit_message>
<xml_diff>
--- a/data/orientation_test_data.xlsx
+++ b/data/orientation_test_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgunda\PlayWright Automation\Projects\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3D0535-7B6B-45D6-93D7-E9CAB104B8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4770150D-165E-40D4-AC72-37F15B011C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
   <si>
     <t>studentEmail</t>
   </si>
@@ -107,12 +107,6 @@
     <t>Test TEST1612</t>
   </si>
   <si>
-    <t>Fall</t>
-  </si>
-  <si>
-    <t>Fall 2026 Orientation</t>
-  </si>
-  <si>
     <t>College of Communication - COM</t>
   </si>
   <si>
@@ -200,14 +194,23 @@
     <t>Cinema &amp; Media Studies|History of Art &amp; Architecture at BU|Arts in Action|Kilachand Honors College: Freedom Trail|BU Marine Program|Finding Your People at BU</t>
   </si>
   <si>
-    <t>Exploring Opportunities at the Pardee School</t>
+    <t>LoginName</t>
+  </si>
+  <si>
+    <t>TEST1612</t>
+  </si>
+  <si>
+    <t>Find Your Squad with First-Year Success</t>
+  </si>
+  <si>
+    <t>TEST2201</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,6 +226,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -265,17 +276,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -576,245 +590,254 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X29"/>
+  <dimension ref="A1:Y29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="22.08984375" customWidth="1"/>
-    <col min="3" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="23" width="22" customWidth="1"/>
-    <col min="24" max="24" width="80" customWidth="1"/>
+    <col min="3" max="3" width="22.08984375" customWidth="1"/>
+    <col min="4" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="8" width="35" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="24" width="22" customWidth="1"/>
+    <col min="25" max="25" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="P2" s="2" t="b">
+      <c r="Q2" s="2" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="T2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="V2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="W2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="X2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="X2" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Y2" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="J3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M3" s="2">
+        <v>72618802</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" s="2">
-        <v>72618802</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="O3" s="2">
+      <c r="P3" s="2">
         <v>92801001</v>
       </c>
-      <c r="P3" s="2" t="b">
+      <c r="Q3" s="2" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="T3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="U3" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="V3" s="2" t="s">
         <v>36</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
-      <c r="C4" s="2"/>
+      <c r="B4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -836,85 +859,87 @@
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P5" s="1"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P6" s="1"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P7" s="1"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P8" s="1"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P9" s="1"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P10" s="1"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P11" s="1"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P12" s="1"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P13" s="1"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P14" s="1"/>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P15" s="1"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="P16" s="1"/>
-    </row>
-    <row r="17" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P17" s="1"/>
-    </row>
-    <row r="18" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P18" s="1"/>
-    </row>
-    <row r="19" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P19" s="1"/>
-    </row>
-    <row r="20" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P20" s="1"/>
-    </row>
-    <row r="21" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P21" s="1"/>
-    </row>
-    <row r="22" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P22" s="1"/>
-    </row>
-    <row r="23" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P23" s="1"/>
-    </row>
-    <row r="24" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P24" s="1"/>
-    </row>
-    <row r="25" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P25" s="1"/>
-    </row>
-    <row r="26" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P26" s="1"/>
-    </row>
-    <row r="27" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P27" s="1"/>
-    </row>
-    <row r="28" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P28" s="1"/>
-    </row>
-    <row r="29" spans="16:16" x14ac:dyDescent="0.35">
-      <c r="P29" s="1"/>
+      <c r="Y4" s="2"/>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q8" s="1"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q9" s="1"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q11" s="1"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q12" s="1"/>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q13" s="1"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q14" s="1"/>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q15" s="1"/>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Q16" s="1"/>
+    </row>
+    <row r="17" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q17" s="1"/>
+    </row>
+    <row r="18" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q18" s="1"/>
+    </row>
+    <row r="19" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q19" s="1"/>
+    </row>
+    <row r="20" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q20" s="1"/>
+    </row>
+    <row r="21" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q21" s="1"/>
+    </row>
+    <row r="22" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q22" s="1"/>
+    </row>
+    <row r="23" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q23" s="1"/>
+    </row>
+    <row r="24" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q24" s="1"/>
+    </row>
+    <row r="25" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q25" s="1"/>
+    </row>
+    <row r="26" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q26" s="1"/>
+    </row>
+    <row r="27" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q27" s="1"/>
+    </row>
+    <row r="28" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q28" s="1"/>
+    </row>
+    <row r="29" spans="17:17" x14ac:dyDescent="0.35">
+      <c r="Q29" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{FBDCC3C5-1B20-49AD-B6A9-4D6DBCD74503}"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{FBDCC3C5-1B20-49AD-B6A9-4D6DBCD74503}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{D6884D97-0164-4F81-AD58-CFCB9CA71ED6}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added changes for code
</commit_message>
<xml_diff>
--- a/data/orientation_test_data.xlsx
+++ b/data/orientation_test_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgunda\PlayWright Automation\Projects\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgunda\PlayWright Automation\BU Test Automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4770150D-165E-40D4-AC72-37F15B011C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FB272-ADE6-463F-B6D8-80639C96D25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -200,10 +200,10 @@
     <t>TEST1612</t>
   </si>
   <si>
-    <t>Find Your Squad with First-Year Success</t>
-  </si>
-  <si>
     <t>TEST2201</t>
+  </si>
+  <si>
+    <t>Exploring Opportunities at the Pardee School</t>
   </si>
 </sst>
 </file>
@@ -751,7 +751,7 @@
         <v>34</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Y2" s="2" t="s">
         <v>52</v>
@@ -762,7 +762,7 @@
         <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>49</v>

</xml_diff>